<commit_message>
Demo bulk file: 4 accounts (2 students, 2 faculty – one BSIT and one BSMEDTECH each)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016PnaiieiWAKMPRCBtnkGwX
</commit_message>
<xml_diff>
--- a/uniroom-admin/templates/demo_bulk_accounts.xlsx
+++ b/uniroom-admin/templates/demo_bulk_accounts.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K9"/>
+  <dimension ref="A1:K5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -550,17 +550,17 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Jessa</t>
+          <t>Kristine</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Villanueva</t>
+          <t>Navarro</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>uniroomsystem+jessa.villanueva@gmail.com</t>
+          <t>uniroomsystem+kristine.navarro@gmail.com</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -569,7 +569,7 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -578,17 +578,17 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>BSIT</t>
+          <t>BSMT</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>BSIT-A1</t>
+          <t>BSMT-A1</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>2026-1002</t>
+          <t>2026-2001</t>
         </is>
       </c>
       <c r="J3" t="inlineStr"/>
@@ -601,17 +601,17 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Mark</t>
+          <t>Ramon</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Aquino</t>
+          <t>Santiago</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>uniroomsystem+mark.aquino@gmail.com</t>
+          <t>uniroomsystem+ramon.santiago@gmail.com</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -620,11 +620,11 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>20</v>
+        <v>41</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>student</t>
+          <t>faculty</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -632,33 +632,33 @@
           <t>BSIT</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>BSIT-A1</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>2026-1003</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr"/>
-      <c r="K4" t="inlineStr"/>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>EMP-2026-01</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>09181110001</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Kristine</t>
+          <t>Teresa</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Navarro</t>
+          <t>Castillo</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>uniroomsystem+kristine.navarro@gmail.com</t>
+          <t>uniroomsystem+teresa.castillo@gmail.com</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -667,11 +667,11 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>19</v>
+        <v>38</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>student</t>
+          <t>faculty</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -679,210 +679,18 @@
           <t>BSMT</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>BSMT-A1</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>2026-2001</t>
-        </is>
-      </c>
-      <c r="J5" t="inlineStr"/>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>EMP-2026-02</t>
+        </is>
+      </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>09171110004</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Joshua</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Mercado</t>
-        </is>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>uniroomsystem+joshua.mercado@gmail.com</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Male</t>
-        </is>
-      </c>
-      <c r="E6" t="n">
-        <v>19</v>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>student</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>BSMT</t>
-        </is>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>BSMT-A2</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>2026-2002</t>
-        </is>
-      </c>
-      <c r="J6" t="inlineStr"/>
-      <c r="K6" t="inlineStr"/>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>Angela</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Dizon</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>uniroomsystem+angela.dizon@gmail.com</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>Female</t>
-        </is>
-      </c>
-      <c r="E7" t="n">
-        <v>20</v>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>student</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>BSMT</t>
-        </is>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>BSMT-A2</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>2026-2003</t>
-        </is>
-      </c>
-      <c r="J7" t="inlineStr"/>
-      <c r="K7" t="inlineStr">
-        <is>
-          <t>09171110006</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>Ramon</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Santiago</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>uniroomsystem+ramon.santiago@gmail.com</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>Male</t>
-        </is>
-      </c>
-      <c r="E8" t="n">
-        <v>41</v>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>faculty</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>BSIT</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr"/>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>EMP-2026-01</t>
-        </is>
-      </c>
-      <c r="K8" t="inlineStr">
-        <is>
-          <t>09181110001</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>Teresa</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Castillo</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>uniroomsystem+teresa.castillo@gmail.com</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>Female</t>
-        </is>
-      </c>
-      <c r="E9" t="n">
-        <v>38</v>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>faculty</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>BSMT</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr"/>
-      <c r="I9" t="inlineStr"/>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t>EMP-2026-02</t>
-        </is>
-      </c>
-      <c r="K9" t="inlineStr"/>
+          <t>09181110002</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>